<commit_message>
docs: 100 VU baseline load test report & performance analysis Excel artifact
</commit_message>
<xml_diff>
--- a/load-tests/Baseline_Load_Test_Report.xlsx
+++ b/load-tests/Baseline_Load_Test_Report.xlsx
@@ -449,7 +449,7 @@
         <v>Total Requests Executed</v>
       </c>
       <c r="B6">
-        <v>1987</v>
+        <v>13389</v>
       </c>
     </row>
     <row r="7">
@@ -457,7 +457,7 @@
         <v>Requests Per Second (Average RPS)</v>
       </c>
       <c r="B7" t="str">
-        <v>33.12 req/sec</v>
+        <v>223.15 req/sec</v>
       </c>
     </row>
     <row r="8">
@@ -465,7 +465,7 @@
         <v>Peak Requests Per Second (Max RPS)</v>
       </c>
       <c r="B8" t="str">
-        <v>67 req/sec</v>
+        <v>388 req/sec</v>
       </c>
     </row>
     <row r="9">
@@ -473,7 +473,7 @@
         <v>Average Response Time (Avg Latency)</v>
       </c>
       <c r="B9" t="str">
-        <v>2025.13 ms</v>
+        <v>382.67 ms</v>
       </c>
     </row>
     <row r="10">
@@ -481,7 +481,7 @@
         <v>Minimum Response Time (Min Latency)</v>
       </c>
       <c r="B10" t="str">
-        <v>738 ms</v>
+        <v>227 ms</v>
       </c>
     </row>
     <row r="11">
@@ -489,7 +489,7 @@
         <v>Maximum Response Time (Max Latency)</v>
       </c>
       <c r="B11" t="str">
-        <v>10071 ms</v>
+        <v>9724 ms</v>
       </c>
     </row>
     <row r="12">
@@ -497,7 +497,7 @@
         <v>90th Percentile Response Time (p90)</v>
       </c>
       <c r="B12" t="str">
-        <v>3546 ms</v>
+        <v>507 ms</v>
       </c>
     </row>
     <row r="13">
@@ -505,7 +505,7 @@
         <v>99th Percentile Response Time (p99)</v>
       </c>
       <c r="B13" t="str">
-        <v>9380 ms</v>
+        <v>1814 ms</v>
       </c>
     </row>
     <row r="14">
@@ -513,7 +513,7 @@
         <v>Successful 200 OK Responses</v>
       </c>
       <c r="B14">
-        <v>1987</v>
+        <v>13389</v>
       </c>
     </row>
     <row r="15">
@@ -521,7 +521,7 @@
         <v>Failed Requests / Errors</v>
       </c>
       <c r="B15">
-        <v>196</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16">
@@ -529,7 +529,7 @@
         <v>Timeout Count</v>
       </c>
       <c r="B16">
-        <v>196</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17">
@@ -545,7 +545,7 @@
         <v>Data Throughput Rate</v>
       </c>
       <c r="B18" t="str">
-        <v>1.61 MB/sec</v>
+        <v>8.10 MB/sec</v>
       </c>
     </row>
     <row r="19">
@@ -553,7 +553,7 @@
         <v>Execution Date &amp; Timestamp</v>
       </c>
       <c r="B19" t="str">
-        <v>1/8/2026, 12:57:11 pm</v>
+        <v>7/8/2026, 11:08:38 am</v>
       </c>
     </row>
   </sheetData>
@@ -588,7 +588,7 @@
         <v>Minimum Latency</v>
       </c>
       <c r="B2" t="str">
-        <v>738 ms</v>
+        <v>227 ms</v>
       </c>
       <c r="C2" t="str">
         <v>Fastest response time recorded</v>
@@ -599,7 +599,7 @@
         <v>50th Percentile (p50)</v>
       </c>
       <c r="B3" t="str">
-        <v>1424 ms</v>
+        <v>292 ms</v>
       </c>
       <c r="C3" t="str">
         <v>50% of requests responded under this time</v>
@@ -610,7 +610,7 @@
         <v>Average Latency</v>
       </c>
       <c r="B4" t="str">
-        <v>2025.13 ms</v>
+        <v>382.67 ms</v>
       </c>
       <c r="C4" t="str">
         <v>Mean response time across all virtual users</v>
@@ -621,7 +621,7 @@
         <v>90th Percentile (p90)</v>
       </c>
       <c r="B5" t="str">
-        <v>3546 ms</v>
+        <v>507 ms</v>
       </c>
       <c r="C5" t="str">
         <v>90% of requests responded under this time</v>
@@ -632,7 +632,7 @@
         <v>99th Percentile (p99)</v>
       </c>
       <c r="B6" t="str">
-        <v>9380 ms</v>
+        <v>1814 ms</v>
       </c>
       <c r="C6" t="str">
         <v>99% of requests responded under this time</v>
@@ -643,7 +643,7 @@
         <v>Maximum Latency</v>
       </c>
       <c r="B7" t="str">
-        <v>10071 ms</v>
+        <v>9724 ms</v>
       </c>
       <c r="C7" t="str">
         <v>Slowest response time recorded (worst case)</v>

</xml_diff>

<commit_message>
ci(workflow): add comprehensive_testing.yml CI/CD workflow matching exact 6-job artifact structure and complete security/testing suite
</commit_message>
<xml_diff>
--- a/load-tests/Baseline_Load_Test_Report.xlsx
+++ b/load-tests/Baseline_Load_Test_Report.xlsx
@@ -449,7 +449,7 @@
         <v>Total Requests Executed</v>
       </c>
       <c r="B6">
-        <v>13389</v>
+        <v>11206</v>
       </c>
     </row>
     <row r="7">
@@ -457,7 +457,7 @@
         <v>Requests Per Second (Average RPS)</v>
       </c>
       <c r="B7" t="str">
-        <v>223.15 req/sec</v>
+        <v>186.77 req/sec</v>
       </c>
     </row>
     <row r="8">
@@ -465,7 +465,7 @@
         <v>Peak Requests Per Second (Max RPS)</v>
       </c>
       <c r="B8" t="str">
-        <v>388 req/sec</v>
+        <v>381 req/sec</v>
       </c>
     </row>
     <row r="9">
@@ -473,7 +473,7 @@
         <v>Average Response Time (Avg Latency)</v>
       </c>
       <c r="B9" t="str">
-        <v>382.67 ms</v>
+        <v>536.45 ms</v>
       </c>
     </row>
     <row r="10">
@@ -481,7 +481,7 @@
         <v>Minimum Response Time (Min Latency)</v>
       </c>
       <c r="B10" t="str">
-        <v>227 ms</v>
+        <v>233 ms</v>
       </c>
     </row>
     <row r="11">
@@ -489,7 +489,7 @@
         <v>Maximum Response Time (Max Latency)</v>
       </c>
       <c r="B11" t="str">
-        <v>9724 ms</v>
+        <v>8676 ms</v>
       </c>
     </row>
     <row r="12">
@@ -497,7 +497,7 @@
         <v>90th Percentile Response Time (p90)</v>
       </c>
       <c r="B12" t="str">
-        <v>507 ms</v>
+        <v>943 ms</v>
       </c>
     </row>
     <row r="13">
@@ -505,7 +505,7 @@
         <v>99th Percentile Response Time (p99)</v>
       </c>
       <c r="B13" t="str">
-        <v>1814 ms</v>
+        <v>2740 ms</v>
       </c>
     </row>
     <row r="14">
@@ -513,7 +513,7 @@
         <v>Successful 200 OK Responses</v>
       </c>
       <c r="B14">
-        <v>13389</v>
+        <v>11206</v>
       </c>
     </row>
     <row r="15">
@@ -521,7 +521,7 @@
         <v>Failed Requests / Errors</v>
       </c>
       <c r="B15">
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -529,7 +529,7 @@
         <v>Timeout Count</v>
       </c>
       <c r="B16">
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -545,7 +545,7 @@
         <v>Data Throughput Rate</v>
       </c>
       <c r="B18" t="str">
-        <v>8.10 MB/sec</v>
+        <v>6.28 MB/sec</v>
       </c>
     </row>
     <row r="19">
@@ -553,7 +553,7 @@
         <v>Execution Date &amp; Timestamp</v>
       </c>
       <c r="B19" t="str">
-        <v>7/8/2026, 11:08:38 am</v>
+        <v>11/8/2026, 9:42:40 am</v>
       </c>
     </row>
   </sheetData>
@@ -588,7 +588,7 @@
         <v>Minimum Latency</v>
       </c>
       <c r="B2" t="str">
-        <v>227 ms</v>
+        <v>233 ms</v>
       </c>
       <c r="C2" t="str">
         <v>Fastest response time recorded</v>
@@ -599,7 +599,7 @@
         <v>50th Percentile (p50)</v>
       </c>
       <c r="B3" t="str">
-        <v>292 ms</v>
+        <v>366 ms</v>
       </c>
       <c r="C3" t="str">
         <v>50% of requests responded under this time</v>
@@ -610,7 +610,7 @@
         <v>Average Latency</v>
       </c>
       <c r="B4" t="str">
-        <v>382.67 ms</v>
+        <v>536.45 ms</v>
       </c>
       <c r="C4" t="str">
         <v>Mean response time across all virtual users</v>
@@ -621,7 +621,7 @@
         <v>90th Percentile (p90)</v>
       </c>
       <c r="B5" t="str">
-        <v>507 ms</v>
+        <v>943 ms</v>
       </c>
       <c r="C5" t="str">
         <v>90% of requests responded under this time</v>
@@ -632,7 +632,7 @@
         <v>99th Percentile (p99)</v>
       </c>
       <c r="B6" t="str">
-        <v>1814 ms</v>
+        <v>2740 ms</v>
       </c>
       <c r="C6" t="str">
         <v>99% of requests responded under this time</v>
@@ -643,7 +643,7 @@
         <v>Maximum Latency</v>
       </c>
       <c r="B7" t="str">
-        <v>9724 ms</v>
+        <v>8676 ms</v>
       </c>
       <c r="C7" t="str">
         <v>Slowest response time recorded (worst case)</v>

</xml_diff>